<commit_message>
Add sourced plant baseline and validation / Ajouter la reference vehicule et sa validation
</commit_message>
<xml_diff>
--- a/docs/verification/BBW_SBW_Requirements_Traceability_EN.xlsx
+++ b/docs/verification/BBW_SBW_Requirements_Traceability_EN.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R3cc4694f342245fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="2" r:id="Rf37b9ed46bb54222"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Catalog" sheetId="3" r:id="Rb5e77df985f843d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R48d35662cc504874"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="2" r:id="R8362ed398a26406d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Catalog" sheetId="3" r:id="Rd4c4584c519540b6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -156,7 +156,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -211,6 +211,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEEAFB"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -347,7 +357,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="123">
+  <x:cellXfs count="126">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -701,11 +711,20 @@
     <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="19">
+  <x:dxfs count="20">
     <x:dxf>
       <x:fill>
         <x:patternFill>
@@ -897,6 +916,17 @@
         </x:patternFill>
       </x:fill>
     </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF087A65"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE2F5F1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
@@ -938,7 +968,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestCatalogTable" displayName="TestCatalogTable" ref="A4:J20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestCatalogTable" displayName="TestCatalogTable" ref="A4:J23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Type"/>
@@ -1555,7 +1585,6 @@
       </x:c>
       <x:c r="I10" s="121" t="str">
         <x:f t="shared" ref="I10:I39" si="1">IF(OR(G10="",H10="",H10&lt;G10),"",H10-G10+1)</x:f>
-        <x:v>Run campaign in MATLAB</x:v>
       </x:c>
       <x:c r="J10" s="84"/>
       <x:c r="K10" s="121" t="str">
@@ -1590,7 +1619,7 @@
       <x:c r="T10" s="13">
         <x:f t="shared" si="2"/>
       </x:c>
-      <x:c r="U10" s="12">
+      <x:c r="U10" s="12" t="str">
         <x:f t="shared" ref="U10:AD19" si="3">IF(OR($G10="",$H10="",$H10&lt;$G10),"",IF(AND(U$9&lt;=$H10,U$9+6&gt;=$G10),1,""))</x:f>
       </x:c>
       <x:c r="V10" s="13">
@@ -2490,7 +2519,7 @@
       <x:c r="T20" s="13">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="U20" s="12">
+      <x:c r="U20" s="12" t="str">
         <x:f t="shared" ref="U20:AD29" si="5">IF(OR($G20="",$H20="",$H20&lt;$G20),"",IF(AND(U$9&lt;=$H20,U$9+6&gt;=$G20),1,""))</x:f>
       </x:c>
       <x:c r="V20" s="13">
@@ -3190,7 +3219,7 @@
         <x:f t="shared" si="1"/>
       </x:c>
       <x:c r="J30" s="102"/>
-      <x:c r="K30" s="12">
+      <x:c r="K30" s="12" t="str">
         <x:f t="shared" ref="K30:T39" si="6">IF(OR($G30="",$H30="",$H30&lt;$G30),"",IF(AND(K$9&lt;=$H30,K$9+6&gt;=$G30),1,""))</x:f>
       </x:c>
       <x:c r="L30" s="13">
@@ -3220,7 +3249,7 @@
       <x:c r="T30" s="13">
         <x:f t="shared" si="6"/>
       </x:c>
-      <x:c r="U30" s="12">
+      <x:c r="U30" s="12" t="str">
         <x:f t="shared" ref="U30:AD39" si="7">IF(OR($G30="",$H30="",$H30&lt;$G30),"",IF(AND(U$9&lt;=$H30,U$9+6&gt;=$G30),1,""))</x:f>
       </x:c>
       <x:c r="V30" s="13">
@@ -4073,7 +4102,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87dcc49348ff4577"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raff3c93dd45f403e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4522,7 +4551,7 @@
         <x:v>G3</x:v>
       </x:c>
       <x:c r="L13" s="95" t="str">
-        <x:v>Current static estimate is 16.6%</x:v>
+        <x:v>Current saturation-limited static estimate is 37.6%</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
@@ -4657,7 +4686,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd16c13c2f8294ee2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re225da820b3f435b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4669,16 +4698,16 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="23" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="40" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="30" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="35" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -4699,7 +4728,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="89" t="str">
-        <x:v>Run validation/run_validation_campaign.m to regenerate results and plots.</x:v>
+        <x:v>Run run_project_validation.m to regenerate plant and allocator evidence.</x:v>
       </x:c>
       <x:c r="B2" s="89"/>
       <x:c r="C2" s="89"/>
@@ -4727,7 +4756,7 @@
       <x:c r="K3" s="90"/>
       <x:c r="L3" s="90"/>
     </x:row>
-    <x:row r="4" ht="28" customHeight="1">
+    <x:row r="4" ht="34" customHeight="1">
       <x:c r="A4" s="93" t="str">
         <x:v>Test ID</x:v>
       </x:c>
@@ -5254,6 +5283,90 @@
       </x:c>
       <x:c r="K20" s="90"/>
       <x:c r="L20" s="90"/>
+    </x:row>
+    <x:row r="21" ht="34" customHeight="1">
+      <x:c r="A21" s="124" t="str">
+        <x:v>PLANT-BRK-01</x:v>
+      </x:c>
+      <x:c r="B21" s="124" t="str">
+        <x:v>Plant</x:v>
+      </x:c>
+      <x:c r="C21" s="124" t="str">
+        <x:v>Symmetric straight-line braking</x:v>
+      </x:c>
+      <x:c r="D21" s="124" t="n">
+        <x:v>-6000</x:v>
+      </x:c>
+      <x:c r="E21" s="124" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F21" s="124" t="str">
+        <x:v>allocator bypassed</x:v>
+      </x:c>
+      <x:c r="G21" s="124"/>
+      <x:c r="H21" s="124" t="str">
+        <x:v>G2 plant</x:v>
+      </x:c>
+      <x:c r="I21" s="124" t="str">
+        <x:v>plant/PLANT-BRK-01/vehicle_response.png</x:v>
+      </x:c>
+      <x:c r="J21" s="124" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="34" customHeight="1">
+      <x:c r="A22" s="125" t="str">
+        <x:v>PLANT-STR-01</x:v>
+      </x:c>
+      <x:c r="B22" s="125" t="str">
+        <x:v>Plant</x:v>
+      </x:c>
+      <x:c r="C22" s="125" t="str">
+        <x:v>Positive one-degree step steer</x:v>
+      </x:c>
+      <x:c r="D22" s="125"/>
+      <x:c r="E22" s="125"/>
+      <x:c r="F22" s="125" t="str">
+        <x:v>allocator bypassed</x:v>
+      </x:c>
+      <x:c r="G22" s="125"/>
+      <x:c r="H22" s="125" t="str">
+        <x:v>G2 plant</x:v>
+      </x:c>
+      <x:c r="I22" s="125" t="str">
+        <x:v>plant/PLANT-STR-01/vehicle_response.png</x:v>
+      </x:c>
+      <x:c r="J22" s="125" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="34" customHeight="1">
+      <x:c r="A23" s="124" t="str">
+        <x:v>PLANT-CMB-01</x:v>
+      </x:c>
+      <x:c r="B23" s="124" t="str">
+        <x:v>Plant</x:v>
+      </x:c>
+      <x:c r="C23" s="124" t="str">
+        <x:v>Combined braking and step steer</x:v>
+      </x:c>
+      <x:c r="D23" s="124" t="n">
+        <x:v>-4000</x:v>
+      </x:c>
+      <x:c r="E23" s="124"/>
+      <x:c r="F23" s="124" t="str">
+        <x:v>allocator bypassed</x:v>
+      </x:c>
+      <x:c r="G23" s="124"/>
+      <x:c r="H23" s="124" t="str">
+        <x:v>G2 plant</x:v>
+      </x:c>
+      <x:c r="I23" s="124" t="str">
+        <x:v>plant/PLANT-CMB-01/vehicle_response.png</x:v>
+      </x:c>
+      <x:c r="J23" s="124" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5265,9 +5378,12 @@
     <x:cfRule type="containsText" dxfId="17" priority="2" operator="containsText" text="Blocked"/>
     <x:cfRule type="containsText" dxfId="18" priority="3" operator="containsText" text="Planned"/>
   </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="J21:J23">
+    <x:cfRule type="containsText" dxfId="19" priority="4" operator="containsText" text="Automated"/>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5362cca75b954931"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87b8249b0b9c48f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>